<commit_message>
Rename the brand from DKKart to DGkart
App name, logo, icons, store graphics, UI text, docs, backend text and the
demo builds now all say DGkart. Example SKUs use a DG- prefix. The demo APK
is also uploaded under its old file name so links already shared still work.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G8cW1vN4fzLnom9wd5TBvX
</commit_message>
<xml_diff>
--- a/docs/samples/image-mapping-template.xlsx
+++ b/docs/samples/image-mapping-template.xlsx
@@ -22,19 +22,19 @@
     <t>position</t>
   </si>
   <si>
-    <t>dk-tshirt-001_1.jpg</t>
-  </si>
-  <si>
-    <t>DK-TSHIRT-001</t>
-  </si>
-  <si>
-    <t>dk-tshirt-001_2.jpg</t>
+    <t>dg-tshirt-001_1.jpg</t>
+  </si>
+  <si>
+    <t>DG-TSHIRT-001</t>
+  </si>
+  <si>
+    <t>dg-tshirt-001_2.jpg</t>
   </si>
   <si>
     <t>earbuds-front.png</t>
   </si>
   <si>
-    <t>DK-EARBUD-002</t>
+    <t>DG-EARBUD-002</t>
   </si>
 </sst>
 </file>

</xml_diff>